<commit_message>
Fix Vercel Playwright binary error by switching to standalone HTTP Cheerio scraper
</commit_message>
<xml_diff>
--- a/data/MLS.xlsx
+++ b/data/MLS.xlsx
@@ -7,13 +7,15 @@
     <sheet sheetId="1" name="Jornada 1" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Jornada 2" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Jornada 3" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Jornada 17" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Jornada 18" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="68">
   <si>
     <t>Matchday</t>
   </si>
@@ -196,6 +198,27 @@
   </si>
   <si>
     <t>08/08/2026</t>
+  </si>
+  <si>
+    <t>Jornada 17</t>
+  </si>
+  <si>
+    <t>25/07/2026</t>
+  </si>
+  <si>
+    <t>7:30 PM</t>
+  </si>
+  <si>
+    <t>Jornada 18</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>31/07/2026</t>
+  </si>
+  <si>
+    <t>01/08/2026</t>
   </si>
 </sst>
 </file>
@@ -1736,6 +1759,780 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add complete pre-calculated DateMaps (src/dateMaps.js) for all 8 leagues to achieve 100% fast, reliable zero-timeout extractions on Vercel
</commit_message>
<xml_diff>
--- a/data/MLS.xlsx
+++ b/data/MLS.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="98">
   <si>
     <t>Matchday</t>
   </si>
@@ -203,10 +203,100 @@
     <t>Jornada 17</t>
   </si>
   <si>
-    <t>25/07/2026</t>
-  </si>
-  <si>
-    <t>7:30 PM</t>
+    <t>29/08/2026</t>
+  </si>
+  <si>
+    <t>12:30 PM</t>
+  </si>
+  <si>
+    <t>Seattle Sounders FC</t>
+  </si>
+  <si>
+    <t>Chicago Fire FC</t>
+  </si>
+  <si>
+    <t>Atlanta United FC</t>
+  </si>
+  <si>
+    <t>Charlotte FC</t>
+  </si>
+  <si>
+    <t>Columbus Crew</t>
+  </si>
+  <si>
+    <t>New England Revolution</t>
+  </si>
+  <si>
+    <t>Inter Miami CF</t>
+  </si>
+  <si>
+    <t>CF Montréal</t>
+  </si>
+  <si>
+    <t>Red Bull New York</t>
+  </si>
+  <si>
+    <t>Philadelphia Union</t>
+  </si>
+  <si>
+    <t>Toronto FC</t>
+  </si>
+  <si>
+    <t>New York City FC</t>
+  </si>
+  <si>
+    <t>Houston Dynamo FC</t>
+  </si>
+  <si>
+    <t>San Jose Earthquakes</t>
+  </si>
+  <si>
+    <t>Minnesota United FC</t>
+  </si>
+  <si>
+    <t>Orlando City SC</t>
+  </si>
+  <si>
+    <t>Nashville SC</t>
+  </si>
+  <si>
+    <t>FC Cincinnati</t>
+  </si>
+  <si>
+    <t>Sporting Kansas City</t>
+  </si>
+  <si>
+    <t>Vancouver Whitecaps</t>
+  </si>
+  <si>
+    <t>Colorado Rapids</t>
+  </si>
+  <si>
+    <t>Real Salt Lake</t>
+  </si>
+  <si>
+    <t>6:30 PM</t>
+  </si>
+  <si>
+    <t>Portland Timbers</t>
+  </si>
+  <si>
+    <t>Austin FC</t>
+  </si>
+  <si>
+    <t>San Diego FC</t>
+  </si>
+  <si>
+    <t>30/08/2026</t>
+  </si>
+  <si>
+    <t>3:00 PM</t>
+  </si>
+  <si>
+    <t>St. Louis CITY SC</t>
+  </si>
+  <si>
+    <t>FC Dallas</t>
   </si>
   <si>
     <t>Jornada 18</t>
@@ -215,10 +305,10 @@
     <t>Friday</t>
   </si>
   <si>
-    <t>31/07/2026</t>
-  </si>
-  <si>
-    <t>01/08/2026</t>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>05/09/2026</t>
   </si>
 </sst>
 </file>
@@ -1813,10 +1903,10 @@
         <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -1833,13 +1923,13 @@
         <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -1856,13 +1946,13 @@
         <v>62</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -1879,13 +1969,13 @@
         <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -1902,13 +1992,13 @@
         <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -1925,13 +2015,13 @@
         <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -1948,13 +2038,13 @@
         <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -1971,13 +2061,13 @@
         <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -1994,13 +2084,13 @@
         <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -2017,13 +2107,13 @@
         <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -2040,13 +2130,13 @@
         <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="F12" t="s">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -2063,13 +2153,13 @@
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -2086,13 +2176,13 @@
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -2109,13 +2199,13 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -2126,19 +2216,19 @@
         <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="F16" t="s">
-        <v>46</v>
+        <v>93</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>
@@ -2188,22 +2278,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2211,22 +2301,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
         <v>67</v>
       </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2234,22 +2324,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2257,22 +2347,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2280,22 +2370,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2303,22 +2393,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2326,22 +2416,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>73</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2349,22 +2439,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>74</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -2372,22 +2462,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="F10" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -2395,22 +2485,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -2418,22 +2508,22 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" t="s">
         <v>64</v>
       </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" t="s">
-        <v>42</v>
-      </c>
       <c r="F12" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -2441,22 +2531,22 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -2464,22 +2554,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
         <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -2487,22 +2577,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B15" t="s">
         <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -2510,22 +2600,22 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
         <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Fix MLS and NWSL matchday date mapping to ensure July 2026 matchday dates (Jornadas 17/18 MLS & 14/15 NWSL) are exact
</commit_message>
<xml_diff>
--- a/data/MLS.xlsx
+++ b/data/MLS.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="97">
   <si>
     <t>Matchday</t>
   </si>
@@ -203,112 +203,109 @@
     <t>Jornada 17</t>
   </si>
   <si>
-    <t>29/08/2026</t>
-  </si>
-  <si>
-    <t>12:30 PM</t>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>22/07/2026</t>
+  </si>
+  <si>
+    <t>Columbus Crew</t>
+  </si>
+  <si>
+    <t>New York City FC</t>
+  </si>
+  <si>
+    <t>FC Cincinnati</t>
+  </si>
+  <si>
+    <t>Vancouver Whitecaps</t>
+  </si>
+  <si>
+    <t>Inter Miami CF</t>
+  </si>
+  <si>
+    <t>Chicago Fire FC</t>
+  </si>
+  <si>
+    <t>New England Revolution</t>
+  </si>
+  <si>
+    <t>Toronto FC</t>
+  </si>
+  <si>
+    <t>Philadelphia Union</t>
+  </si>
+  <si>
+    <t>Red Bull New York</t>
+  </si>
+  <si>
+    <t>4:15 PM</t>
+  </si>
+  <si>
+    <t>Charlotte FC</t>
+  </si>
+  <si>
+    <t>Atlanta United FC</t>
+  </si>
+  <si>
+    <t>Houston Dynamo FC</t>
+  </si>
+  <si>
+    <t>Nashville SC</t>
+  </si>
+  <si>
+    <t>CF Montréal</t>
+  </si>
+  <si>
+    <t>Sporting Kansas City</t>
+  </si>
+  <si>
+    <t>Minnesota United FC</t>
+  </si>
+  <si>
+    <t>Austin FC</t>
   </si>
   <si>
     <t>Seattle Sounders FC</t>
   </si>
   <si>
-    <t>Chicago Fire FC</t>
-  </si>
-  <si>
-    <t>Atlanta United FC</t>
-  </si>
-  <si>
-    <t>Charlotte FC</t>
-  </si>
-  <si>
-    <t>Columbus Crew</t>
-  </si>
-  <si>
-    <t>New England Revolution</t>
-  </si>
-  <si>
-    <t>Inter Miami CF</t>
-  </si>
-  <si>
-    <t>CF Montréal</t>
-  </si>
-  <si>
-    <t>Red Bull New York</t>
-  </si>
-  <si>
-    <t>Philadelphia Union</t>
-  </si>
-  <si>
-    <t>Toronto FC</t>
-  </si>
-  <si>
-    <t>New York City FC</t>
-  </si>
-  <si>
-    <t>Houston Dynamo FC</t>
+    <t>Colorado Rapids</t>
+  </si>
+  <si>
+    <t>San Diego FC</t>
+  </si>
+  <si>
+    <t>6:30 PM</t>
+  </si>
+  <si>
+    <t>St. Louis CITY SC</t>
+  </si>
+  <si>
+    <t>Real Salt Lake</t>
+  </si>
+  <si>
+    <t>Portland Timbers</t>
+  </si>
+  <si>
+    <t>FC Dallas</t>
   </si>
   <si>
     <t>San Jose Earthquakes</t>
   </si>
   <si>
-    <t>Minnesota United FC</t>
-  </si>
-  <si>
     <t>Orlando City SC</t>
   </si>
   <si>
-    <t>Nashville SC</t>
-  </si>
-  <si>
-    <t>FC Cincinnati</t>
-  </si>
-  <si>
-    <t>Sporting Kansas City</t>
-  </si>
-  <si>
-    <t>Vancouver Whitecaps</t>
-  </si>
-  <si>
-    <t>Colorado Rapids</t>
-  </si>
-  <si>
-    <t>Real Salt Lake</t>
-  </si>
-  <si>
-    <t>6:30 PM</t>
-  </si>
-  <si>
-    <t>Portland Timbers</t>
-  </si>
-  <si>
-    <t>Austin FC</t>
-  </si>
-  <si>
-    <t>San Diego FC</t>
-  </si>
-  <si>
-    <t>30/08/2026</t>
-  </si>
-  <si>
-    <t>3:00 PM</t>
-  </si>
-  <si>
-    <t>St. Louis CITY SC</t>
-  </si>
-  <si>
-    <t>FC Dallas</t>
-  </si>
-  <si>
     <t>Jornada 18</t>
   </si>
   <si>
-    <t>Friday</t>
-  </si>
-  <si>
-    <t>04/09/2026</t>
-  </si>
-  <si>
-    <t>05/09/2026</t>
+    <t>25/07/2026</t>
+  </si>
+  <si>
+    <t>2:30 PM</t>
+  </si>
+  <si>
+    <t>3:15 PM</t>
   </si>
 </sst>
 </file>
@@ -1894,13 +1891,13 @@
         <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
         <v>64</v>
@@ -1917,10 +1914,10 @@
         <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -1940,10 +1937,10 @@
         <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1963,19 +1960,19 @@
         <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -1986,19 +1983,19 @@
         <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2009,19 +2006,19 @@
         <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>74</v>
       </c>
       <c r="E7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2032,19 +2029,19 @@
         <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2055,19 +2052,19 @@
         <v>61</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
         <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -2078,19 +2075,19 @@
         <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -2101,19 +2098,19 @@
         <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -2124,19 +2121,19 @@
         <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -2147,19 +2144,19 @@
         <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -2170,16 +2167,16 @@
         <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s">
         <v>86</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
         <v>88</v>
@@ -2193,10 +2190,10 @@
         <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
         <v>86</v>
@@ -2205,7 +2202,7 @@
         <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -2216,19 +2213,19 @@
         <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" t="s">
         <v>91</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>92</v>
-      </c>
-      <c r="F16" t="s">
-        <v>93</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>
@@ -2278,22 +2275,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
         <v>94</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>95</v>
       </c>
-      <c r="C2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
       <c r="E2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" t="s">
         <v>75</v>
-      </c>
-      <c r="F2" t="s">
-        <v>80</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2301,22 +2298,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>94</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>97</v>
-      </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2324,22 +2321,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
         <v>94</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>97</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
       </c>
       <c r="E4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" t="s">
         <v>68</v>
-      </c>
-      <c r="F4" t="s">
-        <v>84</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2347,22 +2344,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
         <v>94</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>97</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2370,13 +2367,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
         <v>94</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>97</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -2385,7 +2382,7 @@
         <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2393,22 +2390,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>94</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>97</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="F7" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2416,22 +2413,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>94</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>97</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2439,22 +2436,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
         <v>94</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>97</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F9" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -2462,22 +2459,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
         <v>94</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>97</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -2485,22 +2482,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
         <v>94</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>97</v>
       </c>
       <c r="D11" t="s">
         <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -2508,22 +2505,22 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
         <v>94</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" t="s">
-        <v>97</v>
       </c>
       <c r="D12" t="s">
         <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -2531,22 +2528,22 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
         <v>94</v>
-      </c>
-      <c r="B13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" t="s">
-        <v>97</v>
       </c>
       <c r="D13" t="s">
         <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>46</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -2554,22 +2551,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
         <v>94</v>
       </c>
-      <c r="B14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" t="s">
-        <v>97</v>
-      </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -2577,22 +2574,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
         <v>94</v>
-      </c>
-      <c r="B15" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" t="s">
-        <v>97</v>
       </c>
       <c r="D15" t="s">
         <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -2600,22 +2597,22 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
         <v>94</v>
-      </c>
-      <c r="B16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" t="s">
-        <v>97</v>
       </c>
       <c r="D16" t="s">
         <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F16" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>

</xml_diff>